<commit_message>
Add productivity, income growth, and demographic dynamics
</commit_message>
<xml_diff>
--- a/simulation_config.xlsx
+++ b/simulation_config.xlsx
@@ -804,7 +804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -968,6 +968,51 @@
       <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Annual %% growth in number of households — new households added each year</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>inflation_target_annual</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Annual baseline inflation target used for normal price drift and transfer indexation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>productivity_growth_rate</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Annual firm productivity growth; raises effective capacity and real wage growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>capital_productivity_multiplier</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Capital income gets this multiple of productivity growth above inflation</t>
         </is>
       </c>
     </row>

</xml_diff>